<commit_message>
f29h85x : mcal: General : Generate release package
- Copy contents from commit ce1803c369f75e93b286f9367d9882e1238b9cd3 in c29x_mcal repo

Signed-off-by: Piyush Panditrao <p-panditrao@ti.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Report/Mcu/TestPlanExecutionReport.xlsx
+++ b/docs/Test_Report/Mcu/TestPlanExecutionReport.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Strategy Compliance'!$A$1:$E$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Plan | Execution Report'!$A$1:$U$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Plan | Execution Report'!$A$1:$U$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +77,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3D3D3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
@@ -104,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -136,13 +131,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -724,7 +716,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990,MCAL-26991</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -734,7 +726,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2024-10-18 10:08:37.673047-05:00 CDT</t>
+          <t>2024-12-18 06:28:58.105926-06:00 CDT</t>
         </is>
       </c>
     </row>
@@ -811,7 +803,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>41</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -826,12 +818,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>41</t>
         </is>
       </c>
     </row>
@@ -848,7 +840,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -863,12 +855,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -885,7 +877,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -905,7 +897,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1025,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>48</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1048,12 +1040,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1116,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1139,7 +1131,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1148,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1171,7 +1163,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1180,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1362,7 +1354,7 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -1372,7 +1364,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="7" t="inlineStr">
@@ -1381,7 +1373,7 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -1391,7 +1383,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
@@ -1409,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U72"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1545,12 +1537,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1657,12 +1649,12 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
@@ -1676,12 +1668,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1788,12 +1780,12 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr"/>
@@ -1807,12 +1799,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1919,12 +1911,12 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr"/>
@@ -1938,12 +1930,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -2050,12 +2042,12 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr"/>
@@ -2069,12 +2061,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2181,12 +2173,12 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr"/>
@@ -2200,12 +2192,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2312,12 +2304,12 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr"/>
@@ -2331,12 +2323,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2443,12 +2435,12 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr"/>
@@ -2462,12 +2454,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2574,12 +2566,12 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr"/>
@@ -2593,12 +2585,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2705,12 +2697,12 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr"/>
@@ -2724,12 +2716,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2836,12 +2828,12 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr"/>
@@ -2855,12 +2847,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -2967,12 +2959,12 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr"/>
@@ -2986,12 +2978,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -3098,12 +3090,12 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S13" s="3" t="inlineStr"/>
@@ -3117,12 +3109,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -3229,12 +3221,12 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
@@ -3248,12 +3240,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -3360,12 +3352,12 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr"/>
@@ -3379,12 +3371,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -3491,12 +3483,12 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr"/>
@@ -3510,12 +3502,12 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -3622,12 +3614,12 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S17" s="3" t="inlineStr"/>
@@ -3641,12 +3633,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -3753,12 +3745,12 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr"/>
@@ -3772,12 +3764,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3884,12 +3876,12 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr"/>
@@ -3903,12 +3895,12 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -4015,12 +4007,12 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr"/>
@@ -4034,12 +4026,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -4146,12 +4138,12 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr"/>
@@ -4165,12 +4157,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -4277,12 +4269,12 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
@@ -4296,12 +4288,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -4408,12 +4400,12 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr"/>
@@ -4427,12 +4419,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -4539,12 +4531,12 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr"/>
@@ -4558,12 +4550,12 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -4670,12 +4662,12 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr"/>
@@ -4689,12 +4681,12 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -4801,12 +4793,12 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
@@ -4820,12 +4812,12 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -4932,12 +4924,12 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
@@ -4951,12 +4943,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -5063,12 +5055,12 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr"/>
@@ -5082,12 +5074,12 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -5194,12 +5186,12 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr"/>
@@ -5213,12 +5205,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -5325,12 +5317,12 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr"/>
@@ -5344,12 +5336,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -5456,12 +5448,12 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr"/>
@@ -5475,12 +5467,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -5587,12 +5579,12 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr"/>
@@ -5606,12 +5598,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -5718,12 +5710,12 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S33" s="3" t="inlineStr"/>
@@ -5737,12 +5729,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5849,12 +5841,12 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S34" s="3" t="inlineStr"/>
@@ -5868,12 +5860,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -5980,12 +5972,12 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S35" s="3" t="inlineStr"/>
@@ -5999,12 +5991,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -6111,12 +6103,12 @@
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S36" s="3" t="inlineStr"/>
@@ -6130,12 +6122,12 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -6242,12 +6234,12 @@
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R37" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S37" s="3" t="inlineStr"/>
@@ -6261,12 +6253,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -6373,12 +6365,12 @@
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R38" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S38" s="3" t="inlineStr"/>
@@ -6392,12 +6384,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -6504,12 +6496,12 @@
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S39" s="3" t="inlineStr"/>
@@ -6523,12 +6515,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -6635,12 +6627,12 @@
       </c>
       <c r="Q40" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R40" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S40" s="3" t="inlineStr"/>
@@ -6654,12 +6646,12 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -6766,12 +6758,12 @@
       </c>
       <c r="Q41" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R41" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S41" s="3" t="inlineStr"/>
@@ -6785,12 +6777,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -6897,12 +6889,12 @@
       </c>
       <c r="Q42" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R42" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S42" s="3" t="inlineStr"/>
@@ -6916,12 +6908,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -7028,12 +7020,12 @@
       </c>
       <c r="Q43" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S43" s="3" t="inlineStr"/>
@@ -7047,12 +7039,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -7159,12 +7151,12 @@
       </c>
       <c r="Q44" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R44" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr"/>
@@ -7178,12 +7170,12 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -7290,12 +7282,12 @@
       </c>
       <c r="Q45" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S45" s="3" t="inlineStr"/>
@@ -7309,12 +7301,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -7421,12 +7413,12 @@
       </c>
       <c r="Q46" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R46" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S46" s="3" t="inlineStr"/>
@@ -7440,12 +7432,12 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -7552,12 +7544,12 @@
       </c>
       <c r="Q47" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr"/>
@@ -7571,12 +7563,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -7683,12 +7675,12 @@
       </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr"/>
@@ -7702,12 +7694,12 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26986</t>
+          <t>MCAL-27998</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>F29H85x - MCAL MCU - Automated Tests</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -7814,12 +7806,12 @@
       </c>
       <c r="Q49" s="3" t="inlineStr">
         <is>
-          <t>MCAL-26990</t>
+          <t>MCAL-27999</t>
         </is>
       </c>
       <c r="R49" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Automated Tests Run</t>
+          <t>F29H85xMCAL_01.01.00 : MCU - Automated Tests Run</t>
         </is>
       </c>
       <c r="S49" s="3" t="inlineStr"/>
@@ -7830,2285 +7822,8 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26973</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_InitClock  test : Clk source: MCU_CLKSRC_XTAL_SE</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21679</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>Choose clock source as  MCU_CLKSRC_XTAL_SE and Mcu_InitClock should not return any DET errors if Mcu_InitClock API is called after  Mcu_Init API and valid clock configuration parameters and valid clock setting ID  are provided</t>
-        </is>
-      </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K50" s="3" t="inlineStr">
-        <is>
-          <t>Check if this API initializes clock settings correctly and returns E_OK std error type and not return any Det and Dem errors</t>
-        </is>
-      </c>
-      <c r="L50" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M50" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N50" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O50" s="3" t="inlineStr">
-        <is>
-          <t>Full,Regression</t>
-        </is>
-      </c>
-      <c r="P50" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q50" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R50" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S50" s="3" t="inlineStr"/>
-      <c r="T50" s="3" t="inlineStr"/>
-      <c r="U50" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26890</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_InitClock  test : Clk source: MCU_CLKSRC_OSC1 : Generate 50 MHZ system clock</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21825,MCAL-21831,MCAL-21834</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>Choose clock source as  MCU_CLKSRC_OSC1 and Mcu_InitClock should not return any DET errors if Mcu_InitClock API is called after  Mcu_Init API and valid clock configuration parameters and valid clock setting ID  are provided</t>
-        </is>
-      </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K51" s="3" t="inlineStr">
-        <is>
-          <t>Check if this API initializes clock settings correctly and returns E_OK std error type and not return any Det and Dem errors</t>
-        </is>
-      </c>
-      <c r="L51" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M51" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N51" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O51" s="3" t="inlineStr">
-        <is>
-          <t>Full,Regression</t>
-        </is>
-      </c>
-      <c r="P51" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q51" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R51" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S51" s="3" t="inlineStr"/>
-      <c r="T51" s="3" t="inlineStr"/>
-      <c r="U51" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26889</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_InitClock  test : Clk source: MCU_CLKSRC_XTAL : Generate 120 MHZ clock</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21825,MCAL-21831,MCAL-21834</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>Choose clock source as  MCU_CLKSRC_XTAL and Mcu_InitClock should not return any DET errors if Mcu_InitClock API is called after  Mcu_Init API and valid clock configuration parameters and valid clock setting ID  are provided</t>
-        </is>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K52" s="3" t="inlineStr">
-        <is>
-          <t>Check if this API initializes clock settings correctly and returns E_OK std error type and not return any Det and Dem errors</t>
-        </is>
-      </c>
-      <c r="L52" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M52" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N52" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O52" s="3" t="inlineStr">
-        <is>
-          <t>Full,Regression</t>
-        </is>
-      </c>
-      <c r="P52" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q52" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R52" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S52" s="3" t="inlineStr"/>
-      <c r="T52" s="3" t="inlineStr"/>
-      <c r="U52" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26394</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>MCU reports development errors and runtime/production errors</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design,Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21793,MCAL-21795,MCAL-21794,MCAL-21850,MCAL-21796,MCAL-21798,MCAL-21797,MCAL-21849</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>Verify if Mcu driver reports development errors and runtime/production errors and use Det-ReportError service and Dem_SetEventStatus</t>
-        </is>
-      </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr">
-        <is>
-          <t>Verify Mcu reports development errors and runtime/production errors</t>
-        </is>
-      </c>
-      <c r="L53" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M53" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N53" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O53" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P53" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q53" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R53" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S53" s="3" t="inlineStr"/>
-      <c r="T53" s="3" t="inlineStr"/>
-      <c r="U53" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26393</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Mcu Module : File Structure</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21784,MCAL-21787,MCAL-21785,MCAL-21786</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>Verify the Mcu driver module file structure is maintained as per autosar SWS document</t>
-        </is>
-      </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr">
-        <is>
-          <t>Verify this test case Manually through code review of  files and folder structure which holds MCU driver module config details and code implementatation and hardware registers information</t>
-        </is>
-      </c>
-      <c r="L54" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M54" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N54" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O54" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P54" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q54" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R54" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S54" s="3" t="inlineStr"/>
-      <c r="T54" s="3" t="inlineStr"/>
-      <c r="U54" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26392</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Testcase to capture ECUC Requirements</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21874,MCAL-21886,MCAL-21902,MCAL-21903,MCAL-21915,MCAL-21918,MCAL-21919,MCAL-23087,MCAL-21859,MCAL-21860,MCAL-21884,MCAL-21892,MCAL-21896,MCAL-21900,MCAL-21906,MCAL-21858,MCAL-21910,MCAL-21911,MCAL-21912,MCAL-21913,MCAL-21930,MCAL-21931,MCAL-21932,MCAL-21935,MCAL-21893,MCAL-21897,MCAL-21861,MCAL-21862,MCAL-21866,MCAL-21880,MCAL-21887,MCAL-21933,MCAL-23088,MCAL-23089,MCAL-23090,MCAL-23092,MCAL-21863,MCAL-21875,MCAL-21876,MCAL-21883,MCAL-21885,MCAL-21894,MCAL-21895,MCAL-21898,MCAL-21904,MCAL-21905,MCAL-21907,MCAL-21937,MCAL-23093,MCAL-21864</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>Verify If the generated tresos configuration files Mcu_Cfg.h and Mcu_PBCfg.c files have data related to all ECUC Requirements</t>
-        </is>
-      </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t>Verify this test case Manually through code review of generated configuration files which holds MCU driver module config details. Check RAM, Clock, Power modes configurations and Pre-compile parameters to enable/disable API's</t>
-        </is>
-      </c>
-      <c r="L55" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M55" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N55" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O55" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P55" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q55" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R55" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S55" s="3" t="inlineStr"/>
-      <c r="T55" s="3" t="inlineStr"/>
-      <c r="U55" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26391</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Qualification Testcase for MCU driver - Reset functionality</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Requirement,Requirement,Requirement,Requirement</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21336,MCAL-21337,MCAL-21338,MCAL-21339</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>Qualification</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver should execute the Reset related functionality i.e Mcu_GetResetReason, Mcu_GetResetRawValue, Mcu_PerformReset API's</t>
-        </is>
-      </c>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K56" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver example Application should sucesdfully call the API's Mcu init, init clock, Get reset raw value and reset reasons and perform reset API's without any DET/DEM/StdErrtype E_NOT_OK errors</t>
-        </is>
-      </c>
-      <c r="L56" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M56" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N56" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O56" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P56" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q56" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R56" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S56" s="3" t="inlineStr"/>
-      <c r="T56" s="3" t="inlineStr"/>
-      <c r="U56" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26390</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Qualification Testcase for MCU driver - Activating reduced power modes</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Requirement,Requirement</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21341,MCAL-21329</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>Qualification</t>
-        </is>
-      </c>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver should execute the low power modes related functionality i.e Mcu_SetMode</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K57" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver example Application should sucessfully call the API's Mcu init, init clock, set mode API's without any DET/DEM/StdErrtype E_NOT_OK errors. After setting inti low power modes, cpu clocks will be gated. So raise an interrupt to ake up from low power modes</t>
-        </is>
-      </c>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M57" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N57" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O57" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P57" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q57" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R57" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S57" s="3" t="inlineStr"/>
-      <c r="T57" s="3" t="inlineStr"/>
-      <c r="U57" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26389</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>Qualification Testcase for MCU driver - Clocking feature</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>Requirement,Requirement,Requirement,Requirement,Requirement,Requirement</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21332,MCAL-23086,MCAL-21335,MCAL-21333,MCAL-21334,MCAL-21340</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>Qualification</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver should execute the Clocking related functionality i.e API's Mcu_InitClock, Mcu_DistributePllClock, Mcu_GetPllStatus</t>
-        </is>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver example Application should sucessfully call the API's Mcu init, init clock, get pll status and distribute pll clock APIs without any DET/DEM/StdErrtype E_NOT_OK errors</t>
-        </is>
-      </c>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M58" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N58" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O58" s="3" t="inlineStr">
-        <is>
-          <t>Full,Regression</t>
-        </is>
-      </c>
-      <c r="P58" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q58" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R58" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S58" s="3" t="inlineStr"/>
-      <c r="T58" s="3" t="inlineStr"/>
-      <c r="U58" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26388</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Qualification Testcase for MCU driver - Ram init and validation features</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Requirement,Requirement</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21331,MCAL-21330</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>Qualification</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver should excute the RAM related functionality i.e API's Mcu_InitRamSection, Mcu_GetRamState</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>MCU driver example Application should sucessfully execute the API's Mcu init, init clock, init ram ad verify ram status without any DET/DEM/StdErrtype E_NOT_OK errors</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N59" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O59" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P59" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S59" s="3" t="inlineStr"/>
-      <c r="T59" s="3" t="inlineStr"/>
-      <c r="U59" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26164</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_PerformReset positive Test</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21684</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_PerformReset should not return any DET errors if Mcu_PerformReset  is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K60" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_PerformReset should not return any DET errors and perform simulation of external reset.</t>
-        </is>
-      </c>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M60" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N60" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O60" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P60" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q60" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R60" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S60" s="3" t="inlineStr"/>
-      <c r="T60" s="3" t="inlineStr"/>
-      <c r="U60" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26163</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode Positive Test: IDLE Mode: Using Xbar Interrupt</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21813,MCAL-21928,MCAL-21941,MCAL-21929,MCAL-21791,MCAL-21792,MCAL-21814,MCAL-21932,MCAL-21877,MCAL-21876,MCAL-21845</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode should not return any DET errors if Mcu_SetMode API is called after  Mcu_Init API and after successful checks of McuMode with Mcu_Mcu_NumberOfLowPowerModes, and also successful checks of mode param config settings</t>
-        </is>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode  API should not return any DET errors</t>
-        </is>
-      </c>
-      <c r="L61" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N61" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O61" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P61" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q61" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R61" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S61" s="3" t="inlineStr"/>
-      <c r="T61" s="3" t="inlineStr"/>
-      <c r="U61" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26162</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode Positive Test:Idle Mode: Using WDG  interrupt</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>Architecture,Architecture,Architecture,Architecture</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21693,MCAL-21688,MCAL-21696,MCAL-21685</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode should not return any DET errors if Mcu_SetMode API is called after  Mcu_Init API and after successful checks of McuMode with Mcu_Mcu_NumberOfLowPowerModes, and also successful checks of mode param config settings</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode  API should not return any DET errors</t>
-        </is>
-      </c>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M62" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N62" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O62" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P62" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q62" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R62" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S62" s="3" t="inlineStr"/>
-      <c r="T62" s="3" t="inlineStr"/>
-      <c r="U62" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26161</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode Positive Test:StandBy Mode: Mcu_EnableWDWakeup flag as True using WDINT</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21941,MCAL-21791,MCAL-21814,MCAL-21877,MCAL-21876,MCAL-21928,MCAL-21845,MCAL-21932,MCAL-21929,MCAL-21792,MCAL-21813,MCAL-21903</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode should not return any DET errors if Mcu_SetMode API is called after  Mcu_Init API and after successful checks of McuMode with Mcu_Mcu_NumberOfLowPowerModes, and also successful checks of mode param config settings</t>
-        </is>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_SetMode  API should not return any DET errors</t>
-        </is>
-      </c>
-      <c r="L63" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M63" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N63" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O63" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P63" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q63" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R63" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S63" s="3" t="inlineStr"/>
-      <c r="T63" s="3" t="inlineStr"/>
-      <c r="U63" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26160</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_ESM_RESET</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21925,MCAL-21919,MCAL-21924</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_ESM_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as MCU_ESM_RESET</t>
-        </is>
-      </c>
-      <c r="L64" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M64" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N64" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O64" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P64" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q64" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R64" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S64" s="3" t="inlineStr"/>
-      <c r="T64" s="3" t="inlineStr"/>
-      <c r="U64" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26159</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_WATCHDOG_RESET</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21925,MCAL-21924,MCAL-21919</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_WATCHDOG_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J65" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as  MCU_WATCHDOG_RESET</t>
-        </is>
-      </c>
-      <c r="L65" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M65" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N65" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O65" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P65" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q65" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R65" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S65" s="3" t="inlineStr"/>
-      <c r="T65" s="3" t="inlineStr"/>
-      <c r="U65" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26158</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_ESM_NMI_WATCHDOG_RESET</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21925,MCAL-21919,MCAL-21924</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_ESM_NMI_WATCHDOG_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K66" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as  MCU_ESM_NMI_WATCHDOG_RESET</t>
-        </is>
-      </c>
-      <c r="L66" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M66" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N66" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O66" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P66" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q66" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R66" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S66" s="3" t="inlineStr"/>
-      <c r="T66" s="3" t="inlineStr"/>
-      <c r="U66" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26157</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_SW_RESET</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21924,MCAL-21789,MCAL-21925,MCAL-21919</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_SW_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J67" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K67" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as  MCU_SW_RESET</t>
-        </is>
-      </c>
-      <c r="L67" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M67" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N67" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O67" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P67" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q67" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R67" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S67" s="3" t="inlineStr"/>
-      <c r="T67" s="3" t="inlineStr"/>
-      <c r="U67" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26156</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_EXTERNAL_RESET</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>Design,Design,Design,Design,Design,Design,Design,Design</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21925,MCAL-21919,MCAL-21789,MCAL-21926,MCAL-21924,MCAL-21809,MCAL-21810,MCAL-21837</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_EXTERNAL_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K68" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as  MCU_EXTERNAL_RESET</t>
-        </is>
-      </c>
-      <c r="L68" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M68" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N68" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O68" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P68" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q68" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R68" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S68" s="3" t="inlineStr"/>
-      <c r="T68" s="3" t="inlineStr"/>
-      <c r="U68" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26155</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason Test : MCU_POWER_ON_RESET</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>Architecture,Architecture</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-21682,MCAL-21691</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>Test case to validate reset reason MCU_POWER_ON_RESET: Mcu_GetResetReason  should not return any DET  if Mcu_GetResetReason  API is called after  Mcu_Init API</t>
-        </is>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>Manual verification</t>
-        </is>
-      </c>
-      <c r="K69" s="3" t="inlineStr">
-        <is>
-          <t>Mcu_GetResetReason  API should not return DET error and return reset reason as  MCU_POWER_ON_RESET</t>
-        </is>
-      </c>
-      <c r="L69" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M69" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N69" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O69" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P69" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q69" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R69" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S69" s="3" t="inlineStr"/>
-      <c r="T69" s="3" t="inlineStr"/>
-      <c r="U69" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-27026</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>Manual Test To verify Mcu Header File inclusions to satisfy AUTOSAR 4.3.1 requirements</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-27021</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t>Manually verify all header files required for Mcu driver are included correctly as per Autosar 4.3.1 requirements</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t>Manual Verification</t>
-        </is>
-      </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t>All header files required for Mcu driver are included correctly as per Autosar 4.3.1 requirements</t>
-        </is>
-      </c>
-      <c r="L70" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M70" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N70" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O70" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P70" s="3" t="inlineStr">
-        <is>
-          <t>Mcu</t>
-        </is>
-      </c>
-      <c r="Q70" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R70" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S70" s="3" t="inlineStr"/>
-      <c r="T70" s="3" t="inlineStr"/>
-      <c r="U70" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-27032</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>Manual Test To Verify AUTOSAR 4.3.1 BSW and SPAL requirements</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture,Architecture</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-12327,MCAL-12305,MCAL-25467,MCAL-12412,MCAL-12411,MCAL-12410,MCAL-12389,MCAL-12374,MCAL-12355,MCAL-12309,MCAL-12448,MCAL-12395,MCAL-12379,MCAL-12375,MCAL-12446,MCAL-25460,MCAL-25458,MCAL-12345,MCAL-12341,MCAL-12356,MCAL-12338,MCAL-12335,MCAL-12333,MCAL-12332,MCAL-12427,MCAL-12421,MCAL-12418,MCAL-25456,MCAL-12376,MCAL-12340,MCAL-12316,MCAL-12312,MCAL-12310,MCAL-12361,MCAL-12399,MCAL-25455,MCAL-25471,MCAL-25469,MCAL-25461,MCAL-12337,MCAL-12334,MCAL-12323,MCAL-12303,MCAL-12425,MCAL-12447,MCAL-12438,MCAL-12444,MCAL-12357,MCAL-12330,MCAL-25464</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t>Manually verify all Modules Design requirements are satisfying the AUTOSAR BSW and SPAL requirements</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t>Manual Verification</t>
-        </is>
-      </c>
-      <c r="K71" s="3" t="inlineStr">
-        <is>
-          <t>Module Design requirements are satisfying the AUTOSAR BSW and SPAL requirements</t>
-        </is>
-      </c>
-      <c r="L71" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M71" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N71" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O71" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P71" s="3" t="inlineStr">
-        <is>
-          <t>Can,Dio,Gpt,Mcu,Port</t>
-        </is>
-      </c>
-      <c r="Q71" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S71" s="3" t="inlineStr"/>
-      <c r="T71" s="3" t="inlineStr"/>
-      <c r="U71" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26987</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-27033</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Manual Test To Verify AUTOSAR 4.3.1 Functional requirement</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>Requirement,Requirement,Requirement,Requirement</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26907,MCAL-26985,MCAL-26908,MCAL-27018</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>F29H85x-evm,F29P58x-evm</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>Qualification</t>
-        </is>
-      </c>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t>Manually verify AUTOSAR 4.3.1 Functional requirement.</t>
-        </is>
-      </c>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t>Manual Verification</t>
-        </is>
-      </c>
-      <c r="K72" s="3" t="inlineStr">
-        <is>
-          <t>AUTOSAR 4.3.1 Requirements are satisfied</t>
-        </is>
-      </c>
-      <c r="L72" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="M72" s="3" t="inlineStr">
-        <is>
-          <t>Requirements-Analysis</t>
-        </is>
-      </c>
-      <c r="N72" s="3" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="O72" s="3" t="inlineStr">
-        <is>
-          <t>Full,Sanity</t>
-        </is>
-      </c>
-      <c r="P72" s="3" t="inlineStr">
-        <is>
-          <t>Port</t>
-        </is>
-      </c>
-      <c r="Q72" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-26991</t>
-        </is>
-      </c>
-      <c r="R72" s="3" t="inlineStr">
-        <is>
-          <t>F29H85xMCAL_01.00.00 : MCU - Manual Tests Run</t>
-        </is>
-      </c>
-      <c r="S72" s="3" t="inlineStr"/>
-      <c r="T72" s="3" t="inlineStr"/>
-      <c r="U72" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:U72"/>
+  <autoFilter ref="A1:U49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10157,12 +7872,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Test Plan</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Test Plan Key</t>
         </is>
@@ -10184,8 +7899,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="n"/>
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Test Plan Name</t>
         </is>
@@ -10207,8 +7922,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n"/>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Test Case Key</t>
         </is>
@@ -10230,8 +7945,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n"/>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Test Case Name</t>
         </is>
@@ -10253,8 +7968,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) Type</t>
         </is>
@@ -10281,8 +7996,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) ID(s)</t>
         </is>
@@ -10304,8 +8019,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Test Platform</t>
         </is>
@@ -10327,8 +8042,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Test Level</t>
         </is>
@@ -10344,7 +8059,7 @@
 -- "Not Provided" if no 'Test Scope' is provided in Jira</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10356,8 +8071,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Test Description</t>
         </is>
@@ -10379,8 +8094,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Test Setup</t>
         </is>
@@ -10402,8 +8117,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Pass/Fail Criteria</t>
         </is>
@@ -10425,8 +8140,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Test Type</t>
         </is>
@@ -10437,7 +8152,7 @@
 (Map Test Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10449,15 +8164,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="13" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Functional:
 Tests covering functional requirements-based  aspects of the software</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10469,8 +8184,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="13" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="12" t="n"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Compatability:
@@ -10478,7 +8193,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing that measures the degree to which a test item can function satisfactorily alongside other independent products in a shared environment (co-existence), and where necessary, exchanges information with other systems or components (interoperability)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10490,15 +8205,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="13" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Usability:
 Test Case covers usability/api/look and feel aspects of the module including out-of box (OOB) experience</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10510,15 +8225,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="12" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Fault Injection:
 Testing based on injection of errors or faults to ensure no unintended consequences</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10530,8 +8245,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="13" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="12" t="n"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Performance: 
@@ -10539,7 +8254,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item accomplishes its designated functions within given constraints of time and other resources</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10551,8 +8266,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="13" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="12" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Reliability: 
@@ -10560,7 +8275,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ability of a test item to perform its required functions, including evaluating the frequency with which failures occur, when it is used under stated conditions for a specified period of time</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10572,8 +8287,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="13" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="12" t="n"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Stress:
@@ -10581,7 +8296,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of performance efficiency testing conducted to evaluate a test item's behaviour under conditions of loading above anticipated or specified capacity requirements, or of resource availability below minimum specified requirements</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10593,8 +8308,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="13" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="12" t="n"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Security:
@@ -10602,7 +8317,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item, and associated data and information, are protected so that unauthorized persons or systems cannot use, read, or modify them, and authorized persons or systems are not denied access to them</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10614,8 +8329,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="13" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="12" t="n"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Maintainability:
@@ -10623,7 +8338,7 @@
 ISO/IEC/IEEE 29119-1 Defn: test type conducted to evaluate the degree of effectiveness and efficiency with which a test item may be modified</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10635,8 +8350,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="13" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="12" t="n"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Portability:
@@ -10644,7 +8359,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ease with which a test item can be transferred from one hardware or software environment to another, including the level of modification needed for it to be executed in various types of environment</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10656,8 +8371,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Test Design Technique</t>
         </is>
@@ -10669,7 +8384,7 @@
 (Map Test Derivation Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10681,8 +8396,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="12" t="n"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Requirements-Analysis:
@@ -10690,7 +8405,7 @@
 </t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10702,15 +8417,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="12" t="n"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Boundary Value Analysis:
 Test cases that apply to interfaces and values approaching and crossing the boundaries and out of range values</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10722,15 +8437,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="13" t="n"/>
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="12" t="n"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Error Guessing:
 Test cases established based on lessons learned and expert judgement to determine situations that may cause software failures or errors to appear</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10742,28 +8457,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Other (Use case analysis; Customer Usage; Requirement analysis; Failure Mode analysis):
 Teams are encouraged to use techniques defined by standards such as ISO/IEC/IEEE 29119-4; which needs to be refelcted within Qmetry</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Test Execution Type</t>
         </is>
@@ -10773,7 +8488,7 @@
           <t>Identifies whether the case is automated or manually or Semi-Automated executed</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10785,8 +8500,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Test Category</t>
         </is>
@@ -10796,7 +8511,7 @@
           <t>Test Categories represent sets of tests that are commonly used.</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10808,15 +8523,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Sanity:
 This Test case is identified to run for Sanity Checks. These are mainly the basic tests that need to be run as part of entry to validate phase</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10828,15 +8543,15 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Full:
 This category means running all test cases for identified releases</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10848,15 +8563,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
-      <c r="B33" s="13" t="n"/>
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="12" t="n"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Base Regression:
 This Test case is identified to run for the Base Regression / maintenance releases</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -10868,8 +8583,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Test Component(s)</t>
         </is>
@@ -10879,24 +8594,24 @@
           <t xml:space="preserve">The field provides the Component(s) (in Jira) to which the Test Case is mapped to. </t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>Test Execution</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Build/Release Key</t>
         </is>
@@ -10918,8 +8633,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Defect Key</t>
         </is>
@@ -10941,8 +8656,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="A37" s="13" t="n"/>
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Defect Summary</t>
         </is>
@@ -10964,8 +8679,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="A38" s="13" t="n"/>
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Overall Status</t>
         </is>
@@ -10988,8 +8703,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
-      <c r="B39" s="13" t="n"/>
+      <c r="A39" s="13" t="n"/>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>PASS
@@ -11008,8 +8723,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="n"/>
-      <c r="B40" s="13" t="n"/>
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="12" t="n"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>FAIL
@@ -11028,8 +8743,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
-      <c r="B41" s="13" t="n"/>
+      <c r="A41" s="13" t="n"/>
+      <c r="B41" s="12" t="n"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>BLOCKED
@@ -11048,8 +8763,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="n"/>
-      <c r="B42" s="13" t="n"/>
+      <c r="A42" s="13" t="n"/>
+      <c r="B42" s="12" t="n"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>WIP

</xml_diff>